<commit_message>
ZLT1: equipmentClass gains dial_gauge and pressure_gauge
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
@@ -1845,9 +1845,21 @@
         <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="19" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>dial_gauge</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>Dial gauge</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>A mechanical or digital indicator that reads a displacement directly, mounted on a reference beam to measure the settlement of a test plate or pile head.</t>
+        </is>
+      </c>
       <c r="E33" s="18" t="n"/>
       <c r="F33" s="18" t="n"/>
       <c r="G33" s="9" t="n"/>
@@ -1857,9 +1869,21 @@
         <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="19" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>pressure_gauge</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Pressure gauge</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>A gauge that reads fluid pressure, for example the Bourdon-tube gauge on a hydraulic jack that gives the load applied in a static load test.</t>
+        </is>
+      </c>
       <c r="E34" s="18" t="n"/>
       <c r="F34" s="18" t="n"/>
       <c r="G34" s="9" t="n"/>
@@ -2442,14 +2466,32 @@
         <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>dial_gauge</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
         <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>pressure_gauge</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35">

</xml_diff>

<commit_message>
PIT2: equipmentClass accelerometer also binds to Equipment/class
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
@@ -2498,7 +2498,16 @@
         <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>accelerometer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36">

</xml_diff>